<commit_message>
Link jobs back to majors in DW schema
</commit_message>
<xml_diff>
--- a/V1.0需求（2026.6.11）/官方数据/DW_专业建设数据模型设计_岗位所属行业更新.xlsx
+++ b/V1.0需求（2026.6.11）/官方数据/DW_专业建设数据模型设计_岗位所属行业更新.xlsx
@@ -2,28 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_总览" sheetId="1" r:id="R87df9525d9e349cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_专业库" sheetId="2" r:id="R3af34b0bf9564d6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_行业库" sheetId="3" r:id="R99323a3891e24af2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_产业链库" sheetId="4" r:id="R5e0c96d8d982400f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_产业环节库" sheetId="5" r:id="Rb40c7d4c75314209"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04A_产业环节关系库" sheetId="6" r:id="R0ea90bfe2e714969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_职业库" sheetId="7" r:id="R189167a99d064858"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_岗位库" sheetId="8" r:id="Rf655683dadf4485d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06A_岗位资源匹配库" sheetId="9" r:id="R8a53c251a7284d01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_岗位任务库" sheetId="10" r:id="R759d9ad0b02f48d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_岗位能力库" sheetId="11" r:id="R08461603aa684a88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_企业库" sheetId="12" r:id="R266c169e8a174faf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_招聘信息库" sheetId="13" r:id="R684342c0dea740fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_招聘趋势库" sheetId="14" r:id="Ra452bf7a47c14866"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11A_新技术岗位匹配库" sheetId="15" r:id="R74c0aea720304ab9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_赛事库" sheetId="16" r:id="R4b933eca33a64e42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_证书库" sheetId="17" r:id="R5182bdcc9c254fec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_课程库" sheetId="18" r:id="R74e94268d3f44d0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_政策库" sheetId="19" r:id="R009737da634f46cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_初始化批次库" sheetId="20" r:id="R0162b8ed7ec14633"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_数据来源目录" sheetId="21" r:id="R287e6876a16f4320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_关联关系" sheetId="22" r:id="R1fb86b84758e4ec4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_总览" sheetId="1" r:id="R5abb546ba9fc4819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_专业库" sheetId="2" r:id="R94a1f6cb5dc5460f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_行业库" sheetId="3" r:id="Rdf68abdb6f19499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_产业链库" sheetId="4" r:id="R92cb92efa93d454e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_产业环节库" sheetId="5" r:id="Rf1daf925ac3b4363"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04A_产业环节关系库" sheetId="6" r:id="R3ee7882868d44aad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_职业库" sheetId="7" r:id="R759da5c4d8554534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_岗位库" sheetId="8" r:id="Rb0e7ec3f3b7349ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06A_岗位资源匹配库" sheetId="9" r:id="R48875828199b46d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_岗位任务库" sheetId="10" r:id="R872ed653ce01413b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_岗位能力库" sheetId="11" r:id="R037d1aa6446d42ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_企业库" sheetId="12" r:id="Ra5567f36293245ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_招聘信息库" sheetId="13" r:id="Re264dc07a33e4e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_招聘趋势库" sheetId="14" r:id="R14b1358879a64c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11A_新技术岗位匹配库" sheetId="15" r:id="R1532367684cf4776"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_赛事库" sheetId="16" r:id="Rcb0faca6bb824d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_证书库" sheetId="17" r:id="R371652958b6a4239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_课程库" sheetId="18" r:id="Rc8fdb166ed704982"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_政策库" sheetId="19" r:id="Rf4486ce65ab946d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_初始化批次库" sheetId="20" r:id="R4f8f2b3058124683"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_数据来源目录" sheetId="21" r:id="R0e2865f7ec484b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_关联关系" sheetId="22" r:id="Rb96367881c3c464b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6652,90 +6652,90 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="11" t="str">
-        <x:v>rel_job_task</x:v>
+        <x:v>rel_job_major</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
         <x:v>岗位</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
-        <x:v>岗位任务</x:v>
+        <x:v>专业</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
-        <x:v>1:N</x:v>
+        <x:v>N:M</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
-        <x:v>job_id -&gt; task_id</x:v>
+        <x:v>related_major_codes -&gt; major_code</x:v>
       </x:c>
       <x:c r="F10" s="11" t="str">
-        <x:v>岗位详情中的典型工作任务。</x:v>
+        <x:v>岗位画像可直接关联多个专业，用于从岗位侧回溯专业建设对象。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="11" t="str">
-        <x:v>rel_job_ability</x:v>
+        <x:v>rel_job_task</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
         <x:v>岗位</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
-        <x:v>岗位能力</x:v>
+        <x:v>岗位任务</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
         <x:v>1:N</x:v>
       </x:c>
       <x:c r="E11" s="11" t="str">
-        <x:v>job_id -&gt; ability_id</x:v>
+        <x:v>job_id -&gt; task_id</x:v>
       </x:c>
       <x:c r="F11" s="11" t="str">
-        <x:v>岗位知识、技能、素养能力项。</x:v>
+        <x:v>岗位详情中的典型工作任务。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="11" t="str">
-        <x:v>rel_task_ability</x:v>
+        <x:v>rel_job_ability</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
-        <x:v>岗位任务</x:v>
+        <x:v>岗位</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
         <x:v>岗位能力</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>N:M</x:v>
+        <x:v>1:N</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
-        <x:v>task_id, ability_id</x:v>
+        <x:v>job_id -&gt; ability_id</x:v>
       </x:c>
       <x:c r="F12" s="11" t="str">
-        <x:v>任务需要若干能力支撑，适合拆为关系表。</x:v>
+        <x:v>岗位知识、技能、素养能力项。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="11" t="str">
-        <x:v>rel_job_course</x:v>
+        <x:v>rel_task_ability</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
-        <x:v>岗位</x:v>
+        <x:v>岗位任务</x:v>
       </x:c>
       <x:c r="C13" s="11" t="str">
-        <x:v>课程</x:v>
+        <x:v>岗位能力</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E13" s="11" t="str">
-        <x:v>job_id, course_id</x:v>
+        <x:v>task_id, ability_id</x:v>
       </x:c>
       <x:c r="F13" s="11" t="str">
-        <x:v>课程支撑岗位能力和岗位建设。</x:v>
+        <x:v>任务需要若干能力支撑，适合拆为关系表。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="11" t="str">
-        <x:v>rel_ability_course</x:v>
+        <x:v>rel_job_course</x:v>
       </x:c>
       <x:c r="B14" s="11" t="str">
-        <x:v>岗位能力</x:v>
+        <x:v>岗位</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
         <x:v>课程</x:v>
@@ -6744,449 +6744,469 @@
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E14" s="11" t="str">
-        <x:v>ability_id, course_id</x:v>
+        <x:v>job_id, course_id</x:v>
       </x:c>
       <x:c r="F14" s="11" t="str">
-        <x:v>课程目标映射能力项。</x:v>
+        <x:v>课程支撑岗位能力和岗位建设。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="11" t="str">
-        <x:v>rel_job_certificate</x:v>
+        <x:v>rel_ability_course</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>岗位</x:v>
+        <x:v>岗位能力</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
-        <x:v>证书</x:v>
+        <x:v>课程</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E15" s="11" t="str">
-        <x:v>job_id, certificate_id</x:v>
+        <x:v>ability_id, course_id</x:v>
       </x:c>
       <x:c r="F15" s="11" t="str">
-        <x:v>岗位可推荐多个证书，一个证书适配多个岗位。</x:v>
+        <x:v>课程目标映射能力项。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="11" t="str">
-        <x:v>rel_job_company</x:v>
+        <x:v>rel_job_certificate</x:v>
       </x:c>
       <x:c r="B16" s="11" t="str">
         <x:v>岗位</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
-        <x:v>企业</x:v>
+        <x:v>证书</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E16" s="11" t="str">
-        <x:v>job_id, company_id</x:v>
+        <x:v>job_id, certificate_id</x:v>
       </x:c>
       <x:c r="F16" s="11" t="str">
-        <x:v>企业样本和主要招聘岗位关系。</x:v>
+        <x:v>岗位可推荐多个证书，一个证书适配多个岗位。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="11" t="str">
-        <x:v>rel_resource_job</x:v>
+        <x:v>rel_job_company</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
-        <x:v>岗位资源匹配</x:v>
+        <x:v>岗位</x:v>
       </x:c>
       <x:c r="C17" s="11" t="str">
-        <x:v>岗位</x:v>
+        <x:v>企业</x:v>
       </x:c>
       <x:c r="D17" s="11" t="str">
-        <x:v>N:1</x:v>
+        <x:v>N:M</x:v>
       </x:c>
       <x:c r="E17" s="11" t="str">
-        <x:v>job_id -&gt; job_id</x:v>
+        <x:v>job_id, company_id</x:v>
       </x:c>
       <x:c r="F17" s="11" t="str">
-        <x:v>岗位画像资源匹配归属具体岗位。</x:v>
+        <x:v>企业样本和主要招聘岗位关系。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="11" t="str">
-        <x:v>rel_resource_major</x:v>
+        <x:v>rel_resource_job</x:v>
       </x:c>
       <x:c r="B18" s="11" t="str">
         <x:v>岗位资源匹配</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>专业</x:v>
+        <x:v>岗位</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
-        <x:v>N:M</x:v>
+        <x:v>N:1</x:v>
       </x:c>
       <x:c r="E18" s="11" t="str">
-        <x:v>major_codes -&gt; major_code</x:v>
+        <x:v>job_id -&gt; job_id</x:v>
       </x:c>
       <x:c r="F18" s="11" t="str">
-        <x:v>岗位画像中的对接专业可回溯到专业库。</x:v>
+        <x:v>岗位画像资源匹配归属具体岗位。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="11" t="str">
-        <x:v>rel_resource_certificate</x:v>
+        <x:v>rel_resource_major</x:v>
       </x:c>
       <x:c r="B19" s="11" t="str">
         <x:v>岗位资源匹配</x:v>
       </x:c>
       <x:c r="C19" s="11" t="str">
-        <x:v>证书</x:v>
+        <x:v>专业</x:v>
       </x:c>
       <x:c r="D19" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E19" s="11" t="str">
-        <x:v>certificate_ids -&gt; certificate_id</x:v>
+        <x:v>major_codes -&gt; major_code</x:v>
       </x:c>
       <x:c r="F19" s="11" t="str">
-        <x:v>岗位画像中的推荐证书可回溯到证书库。</x:v>
+        <x:v>岗位画像中的对接专业可回溯到专业库。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="11" t="str">
-        <x:v>rel_resource_company</x:v>
+        <x:v>rel_resource_certificate</x:v>
       </x:c>
       <x:c r="B20" s="11" t="str">
         <x:v>岗位资源匹配</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
-        <x:v>企业</x:v>
+        <x:v>证书</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E20" s="11" t="str">
-        <x:v>company_ids -&gt; company_id</x:v>
+        <x:v>certificate_ids -&gt; certificate_id</x:v>
       </x:c>
       <x:c r="F20" s="11" t="str">
-        <x:v>岗位画像中的相关企业可回溯到企业库。</x:v>
+        <x:v>岗位画像中的推荐证书可回溯到证书库。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="11" t="str">
-        <x:v>rel_resource_ability</x:v>
+        <x:v>rel_resource_company</x:v>
       </x:c>
       <x:c r="B21" s="11" t="str">
         <x:v>岗位资源匹配</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>岗位能力</x:v>
+        <x:v>企业</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str">
-        <x:v>ability_ids -&gt; ability_id</x:v>
+        <x:v>company_ids -&gt; company_id</x:v>
       </x:c>
       <x:c r="F21" s="11" t="str">
-        <x:v>专业、证书、企业推荐依据可追溯到岗位能力项。</x:v>
+        <x:v>岗位画像中的相关企业可回溯到企业库。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="11" t="str">
-        <x:v>rel_resource_course</x:v>
+        <x:v>rel_resource_ability</x:v>
       </x:c>
       <x:c r="B22" s="11" t="str">
         <x:v>岗位资源匹配</x:v>
       </x:c>
       <x:c r="C22" s="11" t="str">
-        <x:v>课程</x:v>
+        <x:v>岗位能力</x:v>
       </x:c>
       <x:c r="D22" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E22" s="11" t="str">
-        <x:v>course_ids -&gt; course_id</x:v>
+        <x:v>ability_ids -&gt; ability_id</x:v>
       </x:c>
       <x:c r="F22" s="11" t="str">
-        <x:v>岗位资源匹配可转译为课程和实训建议。</x:v>
+        <x:v>专业、证书、企业推荐依据可追溯到岗位能力项。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="11" t="str">
-        <x:v>rel_company_industry</x:v>
+        <x:v>rel_resource_course</x:v>
       </x:c>
       <x:c r="B23" s="11" t="str">
-        <x:v>企业</x:v>
+        <x:v>岗位资源匹配</x:v>
       </x:c>
       <x:c r="C23" s="11" t="str">
-        <x:v>行业</x:v>
+        <x:v>课程</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
-        <x:v>N:1</x:v>
+        <x:v>N:M</x:v>
       </x:c>
       <x:c r="E23" s="11" t="str">
-        <x:v>industry_code</x:v>
+        <x:v>course_ids -&gt; course_id</x:v>
       </x:c>
       <x:c r="F23" s="11" t="str">
-        <x:v>企业按国民经济行业分类归类。</x:v>
+        <x:v>岗位资源匹配可转译为课程和实训建议。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="11" t="str">
-        <x:v>rel_posting_job</x:v>
+        <x:v>rel_company_industry</x:v>
       </x:c>
       <x:c r="B24" s="11" t="str">
-        <x:v>招聘信息</x:v>
+        <x:v>企业</x:v>
       </x:c>
       <x:c r="C24" s="11" t="str">
-        <x:v>岗位</x:v>
+        <x:v>行业</x:v>
       </x:c>
       <x:c r="D24" s="11" t="str">
         <x:v>N:1</x:v>
       </x:c>
       <x:c r="E24" s="11" t="str">
-        <x:v>posting_id -&gt; job_id</x:v>
+        <x:v>industry_code</x:v>
       </x:c>
       <x:c r="F24" s="11" t="str">
-        <x:v>原始招聘标题归一到岗位库。</x:v>
+        <x:v>企业按国民经济行业分类归类。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="11" t="str">
-        <x:v>rel_posting_company</x:v>
+        <x:v>rel_posting_job</x:v>
       </x:c>
       <x:c r="B25" s="11" t="str">
         <x:v>招聘信息</x:v>
       </x:c>
       <x:c r="C25" s="11" t="str">
-        <x:v>企业</x:v>
+        <x:v>岗位</x:v>
       </x:c>
       <x:c r="D25" s="11" t="str">
         <x:v>N:1</x:v>
       </x:c>
       <x:c r="E25" s="11" t="str">
-        <x:v>posting_id -&gt; company_id</x:v>
+        <x:v>posting_id -&gt; job_id</x:v>
       </x:c>
       <x:c r="F25" s="11" t="str">
-        <x:v>招聘企业归一到企业库。</x:v>
+        <x:v>原始招聘标题归一到岗位库。</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="11" t="str">
-        <x:v>rel_trend_job</x:v>
+        <x:v>rel_posting_company</x:v>
       </x:c>
       <x:c r="B26" s="11" t="str">
-        <x:v>招聘趋势</x:v>
+        <x:v>招聘信息</x:v>
       </x:c>
       <x:c r="C26" s="11" t="str">
-        <x:v>岗位/产业链/城市</x:v>
+        <x:v>企业</x:v>
       </x:c>
       <x:c r="D26" s="11" t="str">
-        <x:v>聚合</x:v>
+        <x:v>N:1</x:v>
       </x:c>
       <x:c r="E26" s="11" t="str">
-        <x:v>period, chain_id, job_id, city</x:v>
+        <x:v>posting_id -&gt; company_id</x:v>
       </x:c>
       <x:c r="F26" s="11" t="str">
-        <x:v>按周期沉淀趋势统计，避免实时口径漂移。</x:v>
+        <x:v>招聘企业归一到企业库。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="11" t="str">
+        <x:v>rel_trend_job</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="str">
+        <x:v>招聘趋势</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="str">
+        <x:v>岗位/产业链/城市</x:v>
+      </x:c>
+      <x:c r="D27" s="11" t="str">
+        <x:v>聚合</x:v>
+      </x:c>
+      <x:c r="E27" s="11" t="str">
+        <x:v>period, chain_id, job_id, city</x:v>
+      </x:c>
+      <x:c r="F27" s="11" t="str">
+        <x:v>按周期沉淀趋势统计，避免实时口径漂移。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="11" t="str">
         <x:v>rel_tech_chain</x:v>
-      </x:c>
-      <x:c r="B27" s="11" t="str">
-        <x:v>新技术岗位匹配</x:v>
-      </x:c>
-      <x:c r="C27" s="11" t="str">
-        <x:v>产业链</x:v>
-      </x:c>
-      <x:c r="D27" s="11" t="str">
-        <x:v>N:1</x:v>
-      </x:c>
-      <x:c r="E27" s="11" t="str">
-        <x:v>chain_id -&gt; chain_id</x:v>
-      </x:c>
-      <x:c r="F27" s="11" t="str">
-        <x:v>新技术方向归属产业链，用于按链条过滤研判记录。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="24" hidden="0" customHeight="1">
-      <x:c r="A28" s="11" t="str">
-        <x:v>rel_tech_node</x:v>
       </x:c>
       <x:c r="B28" s="11" t="str">
         <x:v>新技术岗位匹配</x:v>
       </x:c>
       <x:c r="C28" s="11" t="str">
-        <x:v>产业环节</x:v>
+        <x:v>产业链</x:v>
       </x:c>
       <x:c r="D28" s="11" t="str">
         <x:v>N:1</x:v>
       </x:c>
       <x:c r="E28" s="11" t="str">
-        <x:v>industry_node_id -&gt; industry_node_id</x:v>
+        <x:v>chain_id -&gt; chain_id</x:v>
       </x:c>
       <x:c r="F28" s="11" t="str">
-        <x:v>新技术方向关联具体产业环节，支撑产业影响分析。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
+        <x:v>新技术方向归属产业链，用于按链条过滤研判记录。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="24" hidden="0" customHeight="1">
       <x:c r="A29" s="11" t="str">
-        <x:v>rel_tech_job</x:v>
+        <x:v>rel_tech_node</x:v>
       </x:c>
       <x:c r="B29" s="11" t="str">
         <x:v>新技术岗位匹配</x:v>
       </x:c>
       <x:c r="C29" s="11" t="str">
-        <x:v>岗位</x:v>
+        <x:v>产业环节</x:v>
       </x:c>
       <x:c r="D29" s="11" t="str">
         <x:v>N:1</x:v>
       </x:c>
       <x:c r="E29" s="11" t="str">
-        <x:v>job_id -&gt; job_id</x:v>
+        <x:v>industry_node_id -&gt; industry_node_id</x:v>
       </x:c>
       <x:c r="F29" s="11" t="str">
-        <x:v>新技术方向关联新增或强化岗位，并可引用岗位职业路径。</x:v>
+        <x:v>新技术方向关联具体产业环节，支撑产业影响分析。</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="11" t="str">
-        <x:v>rel_tech_major</x:v>
+        <x:v>rel_tech_job</x:v>
       </x:c>
       <x:c r="B30" s="11" t="str">
         <x:v>新技术岗位匹配</x:v>
       </x:c>
       <x:c r="C30" s="11" t="str">
-        <x:v>专业</x:v>
+        <x:v>岗位</x:v>
       </x:c>
       <x:c r="D30" s="11" t="str">
-        <x:v>N:M</x:v>
+        <x:v>N:1</x:v>
       </x:c>
       <x:c r="E30" s="11" t="str">
-        <x:v>major_codes -&gt; major_code</x:v>
+        <x:v>job_id -&gt; job_id</x:v>
       </x:c>
       <x:c r="F30" s="11" t="str">
-        <x:v>新技术方向推荐或关联多个专业，用于专业协同建设。</x:v>
+        <x:v>新技术方向关联新增或强化岗位，并可引用岗位职业路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="11" t="str">
-        <x:v>rel_tech_course</x:v>
+        <x:v>rel_tech_major</x:v>
       </x:c>
       <x:c r="B31" s="11" t="str">
         <x:v>新技术岗位匹配</x:v>
       </x:c>
       <x:c r="C31" s="11" t="str">
-        <x:v>课程</x:v>
+        <x:v>专业</x:v>
       </x:c>
       <x:c r="D31" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E31" s="11" t="str">
-        <x:v>course_ids -&gt; course_id</x:v>
+        <x:v>major_codes -&gt; major_code</x:v>
       </x:c>
       <x:c r="F31" s="11" t="str">
-        <x:v>新技术方向转译为课程或实训建议。</x:v>
+        <x:v>新技术方向推荐或关联多个专业，用于专业协同建设。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="11" t="str">
-        <x:v>rel_tech_ability</x:v>
+        <x:v>rel_tech_course</x:v>
       </x:c>
       <x:c r="B32" s="11" t="str">
         <x:v>新技术岗位匹配</x:v>
       </x:c>
       <x:c r="C32" s="11" t="str">
-        <x:v>岗位能力</x:v>
+        <x:v>课程</x:v>
       </x:c>
       <x:c r="D32" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E32" s="11" t="str">
-        <x:v>ability_ids -&gt; ability_id</x:v>
+        <x:v>course_ids -&gt; course_id</x:v>
       </x:c>
       <x:c r="F32" s="11" t="str">
-        <x:v>新技术方向映射到岗位能力项和课程能力目标。</x:v>
+        <x:v>新技术方向转译为课程或实训建议。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="11" t="str">
-        <x:v>rel_tech_trend</x:v>
+        <x:v>rel_tech_ability</x:v>
       </x:c>
       <x:c r="B33" s="11" t="str">
         <x:v>新技术岗位匹配</x:v>
       </x:c>
       <x:c r="C33" s="11" t="str">
-        <x:v>招聘趋势</x:v>
+        <x:v>岗位能力</x:v>
       </x:c>
       <x:c r="D33" s="11" t="str">
-        <x:v>N:1参考</x:v>
+        <x:v>N:M</x:v>
       </x:c>
       <x:c r="E33" s="11" t="str">
-        <x:v>job_id -&gt; job_id</x:v>
+        <x:v>ability_ids -&gt; ability_id</x:v>
       </x:c>
       <x:c r="F33" s="11" t="str">
-        <x:v>紧缺度、薪资区间和人才缺口判断可回溯招聘趋势。</x:v>
+        <x:v>新技术方向映射到岗位能力项和课程能力目标。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="11" t="str">
-        <x:v>rel_competition_major</x:v>
+        <x:v>rel_tech_trend</x:v>
       </x:c>
       <x:c r="B34" s="11" t="str">
-        <x:v>赛事</x:v>
+        <x:v>新技术岗位匹配</x:v>
       </x:c>
       <x:c r="C34" s="11" t="str">
-        <x:v>专业</x:v>
+        <x:v>招聘趋势</x:v>
       </x:c>
       <x:c r="D34" s="11" t="str">
-        <x:v>N:M</x:v>
+        <x:v>N:1参考</x:v>
       </x:c>
       <x:c r="E34" s="11" t="str">
-        <x:v>competition_id, major_code</x:v>
+        <x:v>job_id -&gt; job_id</x:v>
       </x:c>
       <x:c r="F34" s="11" t="str">
-        <x:v>赛项适配专业。</x:v>
+        <x:v>紧缺度、薪资区间和人才缺口判断可回溯招聘趋势。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="11" t="str">
-        <x:v>rel_competition_ability</x:v>
+        <x:v>rel_competition_major</x:v>
       </x:c>
       <x:c r="B35" s="11" t="str">
         <x:v>赛事</x:v>
       </x:c>
       <x:c r="C35" s="11" t="str">
-        <x:v>岗位能力</x:v>
+        <x:v>专业</x:v>
       </x:c>
       <x:c r="D35" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E35" s="11" t="str">
-        <x:v>competition_id, ability_id</x:v>
+        <x:v>competition_id, major_code</x:v>
       </x:c>
       <x:c r="F35" s="11" t="str">
-        <x:v>赛项能力要求转化为课程和实训依据。</x:v>
+        <x:v>赛项适配专业。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="11" t="str">
-        <x:v>rel_policy_context</x:v>
+        <x:v>rel_competition_ability</x:v>
       </x:c>
       <x:c r="B36" s="11" t="str">
-        <x:v>政策</x:v>
+        <x:v>赛事</x:v>
       </x:c>
       <x:c r="C36" s="11" t="str">
-        <x:v>产业链/专业/岗位</x:v>
+        <x:v>岗位能力</x:v>
       </x:c>
       <x:c r="D36" s="11" t="str">
         <x:v>N:M</x:v>
       </x:c>
       <x:c r="E36" s="11" t="str">
+        <x:v>competition_id, ability_id</x:v>
+      </x:c>
+      <x:c r="F36" s="11" t="str">
+        <x:v>赛项能力要求转化为课程和实训依据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="11" t="str">
+        <x:v>rel_policy_context</x:v>
+      </x:c>
+      <x:c r="B37" s="11" t="str">
+        <x:v>政策</x:v>
+      </x:c>
+      <x:c r="C37" s="11" t="str">
+        <x:v>产业链/专业/岗位</x:v>
+      </x:c>
+      <x:c r="D37" s="11" t="str">
+        <x:v>N:M</x:v>
+      </x:c>
+      <x:c r="E37" s="11" t="str">
         <x:v>policy_id + object_id</x:v>
       </x:c>
-      <x:c r="F36" s="11" t="str">
+      <x:c r="F37" s="11" t="str">
         <x:v>政策可关联多个产业、专业和岗位。</x:v>
       </x:c>
     </x:row>
@@ -9272,44 +9292,42 @@
       </x:c>
       <x:c r="J7" s="11" t="str"/>
     </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
+    <x:row r="8" ht="24" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>industry_node_id</x:v>
+        <x:v>related_major_codes</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
-        <x:v>所属产业环节ID</x:v>
+        <x:v>关联专业</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
-        <x:v>string</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
-        <x:v>是</x:v>
-      </x:c>
-      <x:c r="E8" s="11" t="str">
-        <x:v>FK</x:v>
-      </x:c>
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str"/>
       <x:c r="F8" s="11" t="str">
-        <x:v>岗位承接的产业节点。</x:v>
+        <x:v>岗位可对接或支撑的专业代码列表，用于从岗位画像直接回连专业库。</x:v>
       </x:c>
       <x:c r="G8" s="11" t="str">
-        <x:v>node_bim_platform</x:v>
+        <x:v>440301,440304</x:v>
       </x:c>
       <x:c r="H8" s="11" t="str">
-        <x:v>产业环节库</x:v>
+        <x:v>专业库/岗位画像/规则匹配</x:v>
       </x:c>
       <x:c r="I8" s="11" t="str">
-        <x:v>按项目维护</x:v>
+        <x:v>按版本</x:v>
       </x:c>
       <x:c r="J8" s="11" t="str">
-        <x:v>关联04_产业环节库</x:v>
+        <x:v>关联01_专业库.major_code</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>chain_id</x:v>
+        <x:v>industry_node_id</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>所属产业链ID</x:v>
+        <x:v>所属产业环节ID</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
         <x:v>string</x:v>
@@ -9321,27 +9339,27 @@
         <x:v>FK</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
-        <x:v>岗位归属产业链。</x:v>
+        <x:v>岗位承接的产业节点。</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
-        <x:v>chain_platform</x:v>
+        <x:v>node_bim_platform</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>产业链库</x:v>
+        <x:v>产业环节库</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str">
         <x:v>按项目维护</x:v>
       </x:c>
       <x:c r="J9" s="11" t="str">
-        <x:v>关联03_产业链库</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="24" hidden="0" customHeight="1">
+        <x:v>关联04_产业环节库</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>industry_code</x:v>
+        <x:v>chain_id</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>所属行业代码</x:v>
+        <x:v>所属产业链ID</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
         <x:v>string</x:v>
@@ -9353,62 +9371,62 @@
         <x:v>FK</x:v>
       </x:c>
       <x:c r="F10" s="11" t="str">
-        <x:v>岗位所属行业代码，按岗位归属行业映射到国民经济行业分类。</x:v>
+        <x:v>岗位归属产业链。</x:v>
       </x:c>
       <x:c r="G10" s="11" t="str">
-        <x:v>I65</x:v>
+        <x:v>chain_platform</x:v>
       </x:c>
       <x:c r="H10" s="11" t="str">
-        <x:v>行业库/招聘归并/人工维护</x:v>
+        <x:v>产业链库</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str">
-        <x:v>按批次</x:v>
+        <x:v>按项目维护</x:v>
       </x:c>
       <x:c r="J10" s="11" t="str">
-        <x:v>关联02_行业库</x:v>
+        <x:v>关联03_产业链库</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>industry_name</x:v>
+        <x:v>industry_code</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
-        <x:v>所属行业名称</x:v>
+        <x:v>所属行业代码</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
         <x:v>string</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="E11" s="11" t="str">
-        <x:v>IDX</x:v>
+        <x:v>FK</x:v>
       </x:c>
       <x:c r="F11" s="11" t="str">
-        <x:v>岗位所属行业展示名称，冗余自行业库用于页面展示和筛选。</x:v>
+        <x:v>岗位所属行业代码，按岗位归属行业映射到国民经济行业分类。</x:v>
       </x:c>
       <x:c r="G11" s="11" t="str">
-        <x:v>软件和信息技术服务业</x:v>
+        <x:v>I65</x:v>
       </x:c>
       <x:c r="H11" s="11" t="str">
-        <x:v>行业库/规则映射</x:v>
+        <x:v>行业库/招聘归并/人工维护</x:v>
       </x:c>
       <x:c r="I11" s="11" t="str">
         <x:v>按批次</x:v>
       </x:c>
       <x:c r="J11" s="11" t="str">
-        <x:v>冗余展示字段</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+        <x:v>关联02_行业库</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>job_level</x:v>
+        <x:v>industry_name</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
-        <x:v>岗位层级</x:v>
+        <x:v>所属行业名称</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>enum</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
         <x:v>否</x:v>
@@ -9417,127 +9435,131 @@
         <x:v>IDX</x:v>
       </x:c>
       <x:c r="F12" s="11" t="str">
-        <x:v>初级、中级、高级。</x:v>
+        <x:v>岗位所属行业展示名称，冗余自行业库用于页面展示和筛选。</x:v>
       </x:c>
       <x:c r="G12" s="11" t="str">
-        <x:v>中级</x:v>
+        <x:v>软件和信息技术服务业</x:v>
       </x:c>
       <x:c r="H12" s="11" t="str">
-        <x:v>招聘归并/运营维护</x:v>
+        <x:v>行业库/规则映射</x:v>
       </x:c>
       <x:c r="I12" s="11" t="str">
         <x:v>按批次</x:v>
       </x:c>
-      <x:c r="J12" s="11" t="str"/>
+      <x:c r="J12" s="11" t="str">
+        <x:v>冗余展示字段</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>salary_range</x:v>
+        <x:v>job_level</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
-        <x:v>薪资范围</x:v>
+        <x:v>岗位层级</x:v>
       </x:c>
       <x:c r="C13" s="11" t="str">
-        <x:v>string</x:v>
+        <x:v>enum</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="E13" s="11" t="str"/>
+      <x:c r="E13" s="11" t="str">
+        <x:v>IDX</x:v>
+      </x:c>
       <x:c r="F13" s="11" t="str">
-        <x:v>招聘样本统计后的薪资区间。</x:v>
+        <x:v>初级、中级、高级。</x:v>
       </x:c>
       <x:c r="G13" s="11" t="str">
-        <x:v>10K-18K</x:v>
+        <x:v>中级</x:v>
       </x:c>
       <x:c r="H13" s="11" t="str">
-        <x:v>招聘信息库</x:v>
+        <x:v>招聘归并/运营维护</x:v>
       </x:c>
       <x:c r="I13" s="11" t="str">
-        <x:v>月度/批次</x:v>
+        <x:v>按批次</x:v>
       </x:c>
       <x:c r="J13" s="11" t="str"/>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>demand_level</x:v>
+        <x:v>salary_range</x:v>
       </x:c>
       <x:c r="B14" s="11" t="str">
-        <x:v>需求等级</x:v>
+        <x:v>薪资范围</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
-        <x:v>enum</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="E14" s="11" t="str">
-        <x:v>IDX</x:v>
-      </x:c>
+      <x:c r="E14" s="11" t="str"/>
       <x:c r="F14" s="11" t="str">
-        <x:v>高、中、低、待评估。</x:v>
+        <x:v>招聘样本统计后的薪资区间。</x:v>
       </x:c>
       <x:c r="G14" s="11" t="str">
-        <x:v>高</x:v>
+        <x:v>10K-18K</x:v>
       </x:c>
       <x:c r="H14" s="11" t="str">
-        <x:v>招聘趋势库/规则</x:v>
+        <x:v>招聘信息库</x:v>
       </x:c>
       <x:c r="I14" s="11" t="str">
-        <x:v>月度</x:v>
+        <x:v>月度/批次</x:v>
       </x:c>
       <x:c r="J14" s="11" t="str"/>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>demand_volume</x:v>
+        <x:v>demand_level</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>需求量</x:v>
+        <x:v>需求等级</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
-        <x:v>number</x:v>
+        <x:v>enum</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="E15" s="11" t="str"/>
+      <x:c r="E15" s="11" t="str">
+        <x:v>IDX</x:v>
+      </x:c>
       <x:c r="F15" s="11" t="str">
-        <x:v>统计周期内招聘样本量或需求指数。</x:v>
+        <x:v>高、中、低、待评估。</x:v>
       </x:c>
       <x:c r="G15" s="11" t="str">
-        <x:v>2176</x:v>
+        <x:v>高</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>招聘信息库/招聘趋势库</x:v>
+        <x:v>招聘趋势库/规则</x:v>
       </x:c>
       <x:c r="I15" s="11" t="str">
-        <x:v>月度/批次</x:v>
+        <x:v>月度</x:v>
       </x:c>
       <x:c r="J15" s="11" t="str"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>education</x:v>
+        <x:v>demand_volume</x:v>
       </x:c>
       <x:c r="B16" s="11" t="str">
-        <x:v>学历要求</x:v>
+        <x:v>需求量</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
-        <x:v>enum</x:v>
+        <x:v>number</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="E16" s="11" t="str"/>
       <x:c r="F16" s="11" t="str">
-        <x:v>岗位常见学历门槛。</x:v>
+        <x:v>统计周期内招聘样本量或需求指数。</x:v>
       </x:c>
       <x:c r="G16" s="11" t="str">
-        <x:v>大专及以上</x:v>
+        <x:v>2176</x:v>
       </x:c>
       <x:c r="H16" s="11" t="str">
-        <x:v>招聘信息库</x:v>
+        <x:v>招聘信息库/招聘趋势库</x:v>
       </x:c>
       <x:c r="I16" s="11" t="str">
         <x:v>月度/批次</x:v>
@@ -9546,10 +9568,10 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>experience</x:v>
+        <x:v>education</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
-        <x:v>经验要求</x:v>
+        <x:v>学历要求</x:v>
       </x:c>
       <x:c r="C17" s="11" t="str">
         <x:v>enum</x:v>
@@ -9559,10 +9581,10 @@
       </x:c>
       <x:c r="E17" s="11" t="str"/>
       <x:c r="F17" s="11" t="str">
-        <x:v>岗位常见经验要求。</x:v>
+        <x:v>岗位常见学历门槛。</x:v>
       </x:c>
       <x:c r="G17" s="11" t="str">
-        <x:v>1-3年</x:v>
+        <x:v>大专及以上</x:v>
       </x:c>
       <x:c r="H17" s="11" t="str">
         <x:v>招聘信息库</x:v>
@@ -9572,40 +9594,40 @@
       </x:c>
       <x:c r="J17" s="11" t="str"/>
     </x:row>
-    <x:row r="18" ht="24" hidden="0" customHeight="1">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>career_path</x:v>
+        <x:v>experience</x:v>
       </x:c>
       <x:c r="B18" s="11" t="str">
-        <x:v>职业发展路径</x:v>
+        <x:v>经验要求</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>text</x:v>
+        <x:v>enum</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="E18" s="11" t="str"/>
       <x:c r="F18" s="11" t="str">
-        <x:v>从初级到高级或管理方向的发展路径。</x:v>
+        <x:v>岗位常见经验要求。</x:v>
       </x:c>
       <x:c r="G18" s="11" t="str">
-        <x:v>BIM建模员 -&gt; BIM深化设计工程师 -&gt; BIM项目经理</x:v>
+        <x:v>1-3年</x:v>
       </x:c>
       <x:c r="H18" s="11" t="str">
-        <x:v>岗位画像/人工维护</x:v>
+        <x:v>招聘信息库</x:v>
       </x:c>
       <x:c r="I18" s="11" t="str">
-        <x:v>按版本</x:v>
+        <x:v>月度/批次</x:v>
       </x:c>
       <x:c r="J18" s="11" t="str"/>
     </x:row>
     <x:row r="19" ht="24" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>work_summary</x:v>
+        <x:v>career_path</x:v>
       </x:c>
       <x:c r="B19" s="11" t="str">
-        <x:v>工作内容概述</x:v>
+        <x:v>职业发展路径</x:v>
       </x:c>
       <x:c r="C19" s="11" t="str">
         <x:v>text</x:v>
@@ -9615,25 +9637,25 @@
       </x:c>
       <x:c r="E19" s="11" t="str"/>
       <x:c r="F19" s="11" t="str">
-        <x:v>岗位职责摘要。</x:v>
+        <x:v>从初级到高级或管理方向的发展路径。</x:v>
       </x:c>
       <x:c r="G19" s="11" t="str">
-        <x:v>负责模型深化、碰撞检查、工程量提取与协同交付</x:v>
+        <x:v>BIM建模员 -&gt; BIM深化设计工程师 -&gt; BIM项目经理</x:v>
       </x:c>
       <x:c r="H19" s="11" t="str">
-        <x:v>招聘文本/AI生成后审核</x:v>
+        <x:v>岗位画像/人工维护</x:v>
       </x:c>
       <x:c r="I19" s="11" t="str">
         <x:v>按版本</x:v>
       </x:c>
       <x:c r="J19" s="11" t="str"/>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
+    <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>keywords</x:v>
+        <x:v>work_summary</x:v>
       </x:c>
       <x:c r="B20" s="11" t="str">
-        <x:v>关键词</x:v>
+        <x:v>工作内容概述</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
         <x:v>text</x:v>
@@ -9641,52 +9663,80 @@
       <x:c r="D20" s="11" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="E20" s="11" t="str">
-        <x:v>IDX</x:v>
-      </x:c>
+      <x:c r="E20" s="11" t="str"/>
       <x:c r="F20" s="11" t="str">
-        <x:v>岗位能力、工具、场景关键词。</x:v>
+        <x:v>岗位职责摘要。</x:v>
       </x:c>
       <x:c r="G20" s="11" t="str">
-        <x:v>BIM、Revit、碰撞检查</x:v>
+        <x:v>负责模型深化、碰撞检查、工程量提取与协同交付</x:v>
       </x:c>
       <x:c r="H20" s="11" t="str">
-        <x:v>招聘文本/岗位画像</x:v>
+        <x:v>招聘文本/AI生成后审核</x:v>
       </x:c>
       <x:c r="I20" s="11" t="str">
-        <x:v>按批次</x:v>
+        <x:v>按版本</x:v>
       </x:c>
       <x:c r="J20" s="11" t="str"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>source_batch_id</x:v>
+        <x:v>keywords</x:v>
       </x:c>
       <x:c r="B21" s="11" t="str">
-        <x:v>来源批次ID</x:v>
+        <x:v>关键词</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>string</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str">
-        <x:v>FK</x:v>
+        <x:v>IDX</x:v>
       </x:c>
       <x:c r="F21" s="11" t="str">
-        <x:v>岗位来自哪次采集或初始化批次。</x:v>
+        <x:v>岗位能力、工具、场景关键词。</x:v>
       </x:c>
       <x:c r="G21" s="11" t="str">
-        <x:v>batch_202606</x:v>
+        <x:v>BIM、Revit、碰撞检查</x:v>
       </x:c>
       <x:c r="H21" s="11" t="str">
-        <x:v>采集批次库</x:v>
+        <x:v>招聘文本/岗位画像</x:v>
       </x:c>
       <x:c r="I21" s="11" t="str">
         <x:v>按批次</x:v>
       </x:c>
       <x:c r="J21" s="11" t="str"/>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="12" t="str">
+        <x:v>source_batch_id</x:v>
+      </x:c>
+      <x:c r="B22" s="11" t="str">
+        <x:v>来源批次ID</x:v>
+      </x:c>
+      <x:c r="C22" s="11" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D22" s="11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E22" s="11" t="str">
+        <x:v>FK</x:v>
+      </x:c>
+      <x:c r="F22" s="11" t="str">
+        <x:v>岗位来自哪次采集或初始化批次。</x:v>
+      </x:c>
+      <x:c r="G22" s="11" t="str">
+        <x:v>batch_202606</x:v>
+      </x:c>
+      <x:c r="H22" s="11" t="str">
+        <x:v>采集批次库</x:v>
+      </x:c>
+      <x:c r="I22" s="11" t="str">
+        <x:v>按批次</x:v>
+      </x:c>
+      <x:c r="J22" s="11" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>